<commit_message>
TODO 05 POST CLEANUP
</commit_message>
<xml_diff>
--- a/data/och_extractions_only.xlsx
+++ b/data/och_extractions_only.xlsx
@@ -5,16 +5,19 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tamucc-my.sharepoint.com/personal/chris_bird_tamucc_edu/Documents/!students/Ty_Burris_Thesis/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tamucc-my.sharepoint.com/personal/chris_bird_tamucc_edu/Documents/!students/Ty_Burris_Thesis/Data Analysis/och_cross-contam_testing/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="11_96829CC2CC7168FB5C160B2A3BDCC24551288387" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C8561EF0-71C6-48A0-A56D-3BAEB9ED8451}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="11_96829CC2CC7168FB5C160B2A3BDCC24551288387" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{864F9594-8F70-4EFD-8664-49DF404A7E93}"/>
   <bookViews>
-    <workbookView xWindow="8325" yWindow="-29205" windowWidth="18240" windowHeight="28320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="24975" yWindow="-28965" windowWidth="16440" windowHeight="28320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AZ$351</definedName>
+  </definedNames>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
@@ -3894,6 +3897,8 @@
     <col min="1" max="1" width="13.20703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.41796875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.7890625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.83984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.05078125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:52" s="2" customFormat="1" ht="43.2" x14ac:dyDescent="0.55000000000000004">
@@ -24996,6 +25001,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AZ351" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>